<commit_message>
fix: align Phase 1 assumptions with Day 24 gate
</commit_message>
<xml_diff>
--- a/2A202601912_HuynhThiHaiChau_Day24.xlsx
+++ b/2A202601912_HuynhThiHaiChau_Day24.xlsx
@@ -14,7 +14,9 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'1. Assumptions'!$B$2:$G$41</definedName>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'2. Unit Economics'!$B$2:$G$46</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'2. Unit Economics'!$B$2:$G$48</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">'3. P&amp;L &amp; ROI'!$B$20:$AA$33,'3. P&amp;L &amp; ROI'!$B$36:$J$44</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">'3. P&amp;L &amp; ROI'!$B:$B</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -64,6 +66,39 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
+    <comment ref="D8" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Planning assumption: Optimistic 0.5%, Base 0.3%, Pessimistic 0.1% monthly adoption; all three cases stay within the 0.1%-0.5% range in the Day 24 brief.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>57</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>-197</xdr:colOff>
+                <xdr:row>1</xdr:row>
+                <xdr:rowOff>19</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
     <comment ref="D9" authorId="0">
       <text>
         <r>
@@ -72,7 +107,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: VinFast Q2 2025 results reported 394 global showrooms as of 2025-06-30; planning TAM rounded to 500 locations for network expansion. https://vinfastauto.com/vn_en/vinfast-reports-unaudited-second-quarter-2025-financial-results</t>
+          <t xml:space="preserve">Planning assumption: 10,000 automotive retail locations in the broader Southeast Asia market, set at the lower bound required by the Day 24 lab. VinFast's 394 global showrooms as of 2025-06-30 are treated as the initial beachhead, not the entire TAM. https://vinfastauto.com/vn_en/vinfast-reports-unaudited-second-quarter-2025-financial-results</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -229,6 +264,39 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
+    <comment ref="D32" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Planning assumption: 10B VND committed cash reserve. This is the minimum round-number envelope that keeps the Pessimistic runway above the 12-month gate in the 24-month stress test.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>57</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>-197</xdr:colOff>
+                <xdr:row>1</xdr:row>
+                <xdr:rowOff>19</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
     <comment ref="D35" authorId="0">
       <text>
         <r>
@@ -267,7 +335,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="172">
   <si>
     <t xml:space="preserve">Tab 1 — ASSUMPTIONS  /  Giả định đầu vào</t>
   </si>
@@ -308,7 +376,7 @@
     <t xml:space="preserve">%/tháng</t>
   </si>
   <si>
-    <t xml:space="preserve">Tỷ lệ địa điểm trong TAM bắt đầu trả phí mới mỗi tháng; Pessimistic giảm mạnh so với Base</t>
+    <t xml:space="preserve">Tỷ lệ địa điểm trong TAM bắt đầu trả phí mới mỗi tháng: 0,5% / 0,3% / 0,1%, đúng dải của brief</t>
   </si>
   <si>
     <t xml:space="preserve">Total addressable market (số khách tiềm năng)</t>
@@ -317,7 +385,7 @@
     <t xml:space="preserve">khách</t>
   </si>
   <si>
-    <t xml:space="preserve">Planning TAM 500 địa điểm; neo theo 394 showroom toàn cầu của VinFast tại 30/06/2025</t>
+    <t xml:space="preserve">Planning TAM 10.000 điểm bán ô tô tại Đông Nam Á; VinFast là beachhead, không phải toàn bộ TAM</t>
   </si>
   <si>
     <t xml:space="preserve">2. COGS  /  Chi phí biến đổi trên mỗi khách hàng</t>
@@ -407,7 +475,7 @@
     <t xml:space="preserve">Tiền mặt ban đầu (sau khi đã trừ vốn đầu tư)</t>
   </si>
   <si>
-    <t xml:space="preserve">Ngân sách tiền mặt 5 tỷ VND đã được dành cho 24 tháng vận hành</t>
+    <t xml:space="preserve">Mô hình yêu cầu cam kết 10 tỷ VND tiền mặt để kịch bản xấu vẫn có runway trên 12 tháng</t>
   </si>
   <si>
     <t xml:space="preserve">7. Discount Rate  /  Tỷ suất chiết khấu (cho NPV)</t>
@@ -428,7 +496,7 @@
     <t xml:space="preserve">8. Decision Note  /  Ghi chú quyết định</t>
   </si>
   <si>
-    <t xml:space="preserve">ViVi dùng hybrid pricing B2B: phí nền tảng 9 triệu VND/showroom/tháng cộng usage bình quân 1,5 triệu, nên ARPU Base là 10,5 triệu; CAC 45 triệu phản ánh bán hàng có mục tiêu qua mạng lưới đại lý hiện hữu. Với gross margin 61,9%, mô hình cho LTV/CAC 4,81x và payback 6,9 tháng; Pessimistic giảm ARPU/adoption, tăng churn và CAC ít nhất 1,5x, đồng thời kích hoạt cắt scope để giữ runway 12 tháng.</t>
+    <t xml:space="preserve">ViVi dùng hybrid pricing B2B: phí nền tảng 9 triệu VND/showroom/tháng cộng usage bình quân 1,5 triệu, nên ARPU Base là 10,5 triệu. TAM dùng cho bài là 10.000 điểm bán ô tô tại Đông Nam Á; mạng lưới VinFast là nhóm khách hàng đầu tiên. Adoption 0,3%/tháng ở Base tương đương 30 điểm bán mới. Với gross margin 61,9%, LTV/CAC đạt 4,81x và payback 6,9 tháng. Pessimistic hạ adoption còn 0,1%, tăng churn và CAC lên 1,5x Base; 10 tỷ VND tiền mặt giữ runway 14 tháng để nhóm có thời gian cắt scope.</t>
   </si>
   <si>
     <t xml:space="preserve">Tab 2 — UNIT ECONOMICS  /  Kinh tế đơn vị</t>
@@ -573,6 +641,24 @@
   </si>
   <si>
     <t xml:space="preserve">Assumptions!D22:E22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adoption in lab range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumptions!C8:E8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1%-0.5% all cases</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAM in lab range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumptions!C9:E9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10,000-1,000,000</t>
   </si>
   <si>
     <t xml:space="preserve">Pessimistic runway</t>
@@ -1811,13 +1897,13 @@
         <v>11</v>
       </c>
       <c r="C8" s="13" t="n">
-        <v>0.04</v>
+        <v>0.005</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>0.03</v>
+        <v>0.003</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>0.008</v>
+        <v>0.001</v>
       </c>
       <c r="F8" s="11" t="s">
         <v>12</v>
@@ -1831,13 +1917,13 @@
         <v>14</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>500</v>
+        <v>10000</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>500</v>
+        <v>10000</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>500</v>
+        <v>10000</v>
       </c>
       <c r="F9" s="11" t="s">
         <v>15</v>
@@ -2130,13 +2216,13 @@
         <v>45</v>
       </c>
       <c r="C32" s="10" t="n">
-        <v>5000000000</v>
+        <v>10000000000</v>
       </c>
       <c r="D32" s="10" t="n">
-        <v>5000000000</v>
+        <v>10000000000</v>
       </c>
       <c r="E32" s="10" t="n">
-        <v>5000000000</v>
+        <v>10000000000</v>
       </c>
       <c r="F32" s="11" t="s">
         <v>9</v>
@@ -2254,7 +2340,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:G46"/>
+  <dimension ref="B2:G48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="16.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -2859,15 +2945,15 @@
       <c r="B44" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="C44" s="41" t="n">
-        <f aca="false">'3. P&amp;L &amp; ROI'!C40</f>
-        <v>12</v>
-      </c>
-      <c r="D44" s="41" t="n">
-        <v>12</v>
+      <c r="C44" s="38" t="n">
+        <f aca="false">IF(AND(MIN('1. Assumptions'!C8:E8)&gt;=0.001,MAX('1. Assumptions'!C8:E8)&lt;=0.005),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="D44" s="38" t="n">
+        <v>1</v>
       </c>
       <c r="E44" s="40" t="str">
-        <f aca="false">IF(OR(C44="&gt;= 24",IFERROR(C44&gt;=D44,FALSE())),"OK","FAIL")</f>
+        <f aca="false">IF(C44=D44,"OK","FAIL")</f>
         <v>OK</v>
       </c>
       <c r="F44" s="38" t="s">
@@ -2877,18 +2963,62 @@
         <v>104</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="43" t="s">
+    <row r="45" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B45" s="38" t="s">
         <v>105</v>
       </c>
-      <c r="C46" s="43"/>
-      <c r="D46" s="43"/>
-      <c r="E46" s="43" t="str">
-        <f aca="false">IF(COUNTIF(E39:E44,"FAIL")=0,"PASS","FAIL")</f>
+      <c r="C45" s="38" t="n">
+        <f aca="false">IF(AND(MIN('1. Assumptions'!C9:E9)&gt;=10000,MAX('1. Assumptions'!C9:E9)&lt;=1000000),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="D45" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" s="40" t="str">
+        <f aca="false">IF(C45=D45,"OK","FAIL")</f>
+        <v>OK</v>
+      </c>
+      <c r="F45" s="38" t="s">
+        <v>106</v>
+      </c>
+      <c r="G45" s="38" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B46" s="38" t="s">
+        <v>108</v>
+      </c>
+      <c r="C46" s="41" t="n">
+        <f aca="false">'3. P&amp;L &amp; ROI'!C40</f>
+        <v>14</v>
+      </c>
+      <c r="D46" s="41" t="n">
+        <v>12</v>
+      </c>
+      <c r="E46" s="40" t="str">
+        <f aca="false">IF(OR(C46="&gt;= 24",IFERROR(C46&gt;=D46,FALSE())),"OK","FAIL")</f>
+        <v>OK</v>
+      </c>
+      <c r="F46" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="G46" s="38" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B48" s="43" t="s">
+        <v>111</v>
+      </c>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43" t="str">
+        <f aca="false">IF(COUNTIF(E39:E46,"FAIL")=0,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
-      <c r="F46" s="43"/>
-      <c r="G46" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -2902,8 +3032,8 @@
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
     <mergeCell ref="B37:G37"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="E46:G46"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="E48:G48"/>
   </mergeCells>
   <conditionalFormatting sqref="C21">
     <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -3010,7 +3140,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B2:AA44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="16.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -3023,7 +3153,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="30" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3035,13 +3165,13 @@
     <row r="3" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="4" customFormat="false" ht="15" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="44" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C4" s="45" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
@@ -3051,7 +3181,7 @@
     <row r="5" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="6" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="46" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="C6" s="46" t="n">
         <f aca="false">MATCH(C4,{"Optimistic","Base","Pessimistic"},0)</f>
@@ -3060,12 +3190,12 @@
     </row>
     <row r="7" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="47" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="48" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="C8" s="49" t="n">
         <f aca="false">CHOOSE($C$6,'1. Assumptions'!C7,'1. Assumptions'!D7,'1. Assumptions'!E7)</f>
@@ -3074,25 +3204,25 @@
     </row>
     <row r="9" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="48" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C9" s="50" t="n">
         <f aca="false">CHOOSE($C$6,'1. Assumptions'!C8,'1. Assumptions'!D8,'1. Assumptions'!E8)</f>
-        <v>0.008</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="48" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C10" s="49" t="n">
         <f aca="false">CHOOSE($C$6,'1. Assumptions'!C9,'1. Assumptions'!D9,'1. Assumptions'!E9)</f>
-        <v>500</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="48" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="C11" s="49" t="n">
         <f aca="false">CHOOSE($C$6,'1. Assumptions'!C15,'1. Assumptions'!D15,'1. Assumptions'!E15)</f>
@@ -3101,7 +3231,7 @@
     </row>
     <row r="12" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="48" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="C12" s="50" t="n">
         <f aca="false">CHOOSE($C$6,'1. Assumptions'!C18,'1. Assumptions'!D18,'1. Assumptions'!E18)</f>
@@ -3110,7 +3240,7 @@
     </row>
     <row r="13" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="48" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="C13" s="49" t="n">
         <f aca="false">CHOOSE($C$6,'1. Assumptions'!C22,'1. Assumptions'!D22,'1. Assumptions'!E22)</f>
@@ -3119,7 +3249,7 @@
     </row>
     <row r="14" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="48" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="C14" s="49" t="n">
         <f aca="false">CHOOSE($C$6,'1. Assumptions'!C28,'1. Assumptions'!D28,'1. Assumptions'!E28)</f>
@@ -3128,7 +3258,7 @@
     </row>
     <row r="15" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="48" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C15" s="49" t="n">
         <f aca="false">CHOOSE($C$6,'1. Assumptions'!C31,'1. Assumptions'!D31,'1. Assumptions'!E31)</f>
@@ -3137,16 +3267,16 @@
     </row>
     <row r="16" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="48" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="C16" s="49" t="n">
         <f aca="false">CHOOSE($C$6,'1. Assumptions'!C32,'1. Assumptions'!D32,'1. Assumptions'!E32)</f>
-        <v>5000000000</v>
+        <v>10000000000</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="48" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C17" s="50" t="n">
         <f aca="false">CHOOSE($C$6,'1. Assumptions'!C36,'1. Assumptions'!D36,'1. Assumptions'!E36)</f>
@@ -3155,7 +3285,7 @@
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="3" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
@@ -3185,713 +3315,713 @@
     </row>
     <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="51" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C21" s="52" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="D21" s="52" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="E21" s="52" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="F21" s="52" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="G21" s="52" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="H21" s="52" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="I21" s="52" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="J21" s="52" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="K21" s="52" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="L21" s="52" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="M21" s="52" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="N21" s="52" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="O21" s="52" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="P21" s="52" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="Q21" s="52" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="R21" s="52" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="S21" s="52" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="T21" s="52" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="U21" s="52" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="V21" s="52" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="W21" s="52" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="X21" s="52" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="Y21" s="52" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="Z21" s="52" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="AA21" s="53" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="9" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="C22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="I22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="K22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="L22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="M22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="N22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="O22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="P22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="Q22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="R22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="S22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="T22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="U22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="V22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="W22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="X22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="Y22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="Z22" s="54" t="n">
         <f aca="false">ROUND($C$10*$C$9,0)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="AA22" s="55" t="n">
         <f aca="false">SUM(C22:Z22)</f>
-        <v>96</v>
+        <v>240</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="9" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="C23" s="54" t="n">
         <f aca="false">C22</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D23" s="54" t="n">
         <f aca="false">C23*(1-$C$12)+D22</f>
-        <v>7.82</v>
+        <v>19.55</v>
       </c>
       <c r="E23" s="54" t="n">
         <f aca="false">D23*(1-$C$12)+E22</f>
-        <v>11.4681</v>
+        <v>28.67025</v>
       </c>
       <c r="F23" s="54" t="n">
         <f aca="false">E23*(1-$C$12)+F22</f>
-        <v>14.9520355</v>
+        <v>37.38008875</v>
       </c>
       <c r="G23" s="54" t="n">
         <f aca="false">F23*(1-$C$12)+G22</f>
-        <v>18.2791939025</v>
+        <v>45.69798475625</v>
       </c>
       <c r="H23" s="54" t="n">
         <f aca="false">G23*(1-$C$12)+H22</f>
-        <v>21.4566301768875</v>
+        <v>53.6415754422187</v>
       </c>
       <c r="I23" s="54" t="n">
         <f aca="false">H23*(1-$C$12)+I22</f>
-        <v>24.4910818189276</v>
+        <v>61.2277045473189</v>
       </c>
       <c r="J23" s="54" t="n">
         <f aca="false">I23*(1-$C$12)+J22</f>
-        <v>27.3889831370758</v>
+        <v>68.4724578426896</v>
       </c>
       <c r="K23" s="54" t="n">
         <f aca="false">J23*(1-$C$12)+K22</f>
-        <v>30.1564788959074</v>
+        <v>75.3911972397685</v>
       </c>
       <c r="L23" s="54" t="n">
         <f aca="false">K23*(1-$C$12)+L22</f>
-        <v>32.7994373455916</v>
+        <v>81.9985933639789</v>
       </c>
       <c r="M23" s="54" t="n">
         <f aca="false">L23*(1-$C$12)+M22</f>
-        <v>35.32346266504</v>
+        <v>88.3086566625999</v>
       </c>
       <c r="N23" s="54" t="n">
         <f aca="false">M23*(1-$C$12)+N22</f>
-        <v>37.7339068451132</v>
+        <v>94.3347671127829</v>
       </c>
       <c r="O23" s="54" t="n">
         <f aca="false">N23*(1-$C$12)+O22</f>
-        <v>40.0358810370831</v>
+        <v>100.089702592708</v>
       </c>
       <c r="P23" s="54" t="n">
         <f aca="false">O23*(1-$C$12)+P22</f>
-        <v>42.2342663904143</v>
+        <v>105.585665976036</v>
       </c>
       <c r="Q23" s="54" t="n">
         <f aca="false">P23*(1-$C$12)+Q22</f>
-        <v>44.3337244028457</v>
+        <v>110.834311007114</v>
       </c>
       <c r="R23" s="54" t="n">
         <f aca="false">Q23*(1-$C$12)+R22</f>
-        <v>46.3387068047176</v>
+        <v>115.846767011794</v>
       </c>
       <c r="S23" s="54" t="n">
         <f aca="false">R23*(1-$C$12)+S22</f>
-        <v>48.2534649985053</v>
+        <v>120.633662496263</v>
       </c>
       <c r="T23" s="54" t="n">
         <f aca="false">S23*(1-$C$12)+T22</f>
-        <v>50.0820590735726</v>
+        <v>125.205147683931</v>
       </c>
       <c r="U23" s="54" t="n">
         <f aca="false">T23*(1-$C$12)+U22</f>
-        <v>51.8283664152618</v>
+        <v>129.570916038155</v>
       </c>
       <c r="V23" s="54" t="n">
         <f aca="false">U23*(1-$C$12)+V22</f>
-        <v>53.496089926575</v>
+        <v>133.740224816438</v>
       </c>
       <c r="W23" s="54" t="n">
         <f aca="false">V23*(1-$C$12)+W22</f>
-        <v>55.0887658798792</v>
+        <v>137.721914699698</v>
       </c>
       <c r="X23" s="54" t="n">
         <f aca="false">W23*(1-$C$12)+X22</f>
-        <v>56.6097714152846</v>
+        <v>141.524428538211</v>
       </c>
       <c r="Y23" s="54" t="n">
         <f aca="false">X23*(1-$C$12)+Y22</f>
-        <v>58.0623317015968</v>
+        <v>145.155829253992</v>
       </c>
       <c r="Z23" s="54" t="n">
         <f aca="false">Y23*(1-$C$12)+Z22</f>
-        <v>59.4495267750249</v>
+        <v>148.623816937562</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="56" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="C25" s="57" t="n">
         <f aca="false">C23*$C$8</f>
-        <v>32000000</v>
+        <v>80000000</v>
       </c>
       <c r="D25" s="57" t="n">
         <f aca="false">D23*$C$8</f>
-        <v>62560000</v>
+        <v>156400000</v>
       </c>
       <c r="E25" s="57" t="n">
         <f aca="false">E23*$C$8</f>
-        <v>91744800</v>
+        <v>229362000</v>
       </c>
       <c r="F25" s="57" t="n">
         <f aca="false">F23*$C$8</f>
-        <v>119616284</v>
+        <v>299040710</v>
       </c>
       <c r="G25" s="57" t="n">
         <f aca="false">G23*$C$8</f>
-        <v>146233551.22</v>
+        <v>365583878.05</v>
       </c>
       <c r="H25" s="57" t="n">
         <f aca="false">H23*$C$8</f>
-        <v>171653041.4151</v>
+        <v>429132603.53775</v>
       </c>
       <c r="I25" s="57" t="n">
         <f aca="false">I23*$C$8</f>
-        <v>195928654.55142</v>
+        <v>489821636.378551</v>
       </c>
       <c r="J25" s="57" t="n">
         <f aca="false">J23*$C$8</f>
-        <v>219111865.096607</v>
+        <v>547779662.741516</v>
       </c>
       <c r="K25" s="57" t="n">
         <f aca="false">K23*$C$8</f>
-        <v>241251831.167259</v>
+        <v>603129577.918148</v>
       </c>
       <c r="L25" s="57" t="n">
         <f aca="false">L23*$C$8</f>
-        <v>262395498.764733</v>
+        <v>655988746.911831</v>
       </c>
       <c r="M25" s="57" t="n">
         <f aca="false">M23*$C$8</f>
-        <v>282587701.32032</v>
+        <v>706469253.300799</v>
       </c>
       <c r="N25" s="57" t="n">
         <f aca="false">N23*$C$8</f>
-        <v>301871254.760905</v>
+        <v>754678136.902263</v>
       </c>
       <c r="O25" s="57" t="n">
         <f aca="false">O23*$C$8</f>
-        <v>320287048.296664</v>
+        <v>800717620.741661</v>
       </c>
       <c r="P25" s="57" t="n">
         <f aca="false">P23*$C$8</f>
-        <v>337874131.123315</v>
+        <v>844685327.808286</v>
       </c>
       <c r="Q25" s="57" t="n">
         <f aca="false">Q23*$C$8</f>
-        <v>354669795.222765</v>
+        <v>886674488.056913</v>
       </c>
       <c r="R25" s="57" t="n">
         <f aca="false">R23*$C$8</f>
-        <v>370709654.437741</v>
+        <v>926774136.094352</v>
       </c>
       <c r="S25" s="57" t="n">
         <f aca="false">S23*$C$8</f>
-        <v>386027719.988043</v>
+        <v>965069299.970106</v>
       </c>
       <c r="T25" s="57" t="n">
         <f aca="false">T23*$C$8</f>
-        <v>400656472.588581</v>
+        <v>1001641181.47145</v>
       </c>
       <c r="U25" s="57" t="n">
         <f aca="false">U23*$C$8</f>
-        <v>414626931.322094</v>
+        <v>1036567328.30524</v>
       </c>
       <c r="V25" s="57" t="n">
         <f aca="false">V23*$C$8</f>
-        <v>427968719.4126</v>
+        <v>1069921798.5315</v>
       </c>
       <c r="W25" s="57" t="n">
         <f aca="false">W23*$C$8</f>
-        <v>440710127.039033</v>
+        <v>1101775317.59758</v>
       </c>
       <c r="X25" s="57" t="n">
         <f aca="false">X23*$C$8</f>
-        <v>452878171.322277</v>
+        <v>1132195428.30569</v>
       </c>
       <c r="Y25" s="57" t="n">
         <f aca="false">Y23*$C$8</f>
-        <v>464498653.612774</v>
+        <v>1161246634.03194</v>
       </c>
       <c r="Z25" s="57" t="n">
         <f aca="false">Z23*$C$8</f>
-        <v>475596214.200199</v>
+        <v>1188990535.5005</v>
       </c>
       <c r="AA25" s="58" t="n">
         <f aca="false">SUM(C25:Z25)</f>
-        <v>6973458120.86243</v>
+        <v>17433645302.1561</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="9" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C26" s="54" t="n">
         <f aca="false">C23*$C$11</f>
-        <v>20000000</v>
+        <v>50000000</v>
       </c>
       <c r="D26" s="54" t="n">
         <f aca="false">D23*$C$11</f>
-        <v>39100000</v>
+        <v>97750000</v>
       </c>
       <c r="E26" s="54" t="n">
         <f aca="false">E23*$C$11</f>
-        <v>57340500</v>
+        <v>143351250</v>
       </c>
       <c r="F26" s="54" t="n">
         <f aca="false">F23*$C$11</f>
-        <v>74760177.5</v>
+        <v>186900443.75</v>
       </c>
       <c r="G26" s="54" t="n">
         <f aca="false">G23*$C$11</f>
-        <v>91395969.5125</v>
+        <v>228489923.78125</v>
       </c>
       <c r="H26" s="54" t="n">
         <f aca="false">H23*$C$11</f>
-        <v>107283150.884437</v>
+        <v>268207877.211094</v>
       </c>
       <c r="I26" s="54" t="n">
         <f aca="false">I23*$C$11</f>
-        <v>122455409.094638</v>
+        <v>306138522.736595</v>
       </c>
       <c r="J26" s="54" t="n">
         <f aca="false">J23*$C$11</f>
-        <v>136944915.685379</v>
+        <v>342362289.213448</v>
       </c>
       <c r="K26" s="54" t="n">
         <f aca="false">K23*$C$11</f>
-        <v>150782394.479537</v>
+        <v>376955986.198843</v>
       </c>
       <c r="L26" s="54" t="n">
         <f aca="false">L23*$C$11</f>
-        <v>163997186.727958</v>
+        <v>409992966.819895</v>
       </c>
       <c r="M26" s="54" t="n">
         <f aca="false">M23*$C$11</f>
-        <v>176617313.3252</v>
+        <v>441543283.312999</v>
       </c>
       <c r="N26" s="54" t="n">
         <f aca="false">N23*$C$11</f>
-        <v>188669534.225566</v>
+        <v>471673835.563914</v>
       </c>
       <c r="O26" s="54" t="n">
         <f aca="false">O23*$C$11</f>
-        <v>200179405.185415</v>
+        <v>500448512.963538</v>
       </c>
       <c r="P26" s="54" t="n">
         <f aca="false">P23*$C$11</f>
-        <v>211171331.952072</v>
+        <v>527928329.880179</v>
       </c>
       <c r="Q26" s="54" t="n">
         <f aca="false">Q23*$C$11</f>
-        <v>221668622.014228</v>
+        <v>554171555.035571</v>
       </c>
       <c r="R26" s="54" t="n">
         <f aca="false">R23*$C$11</f>
-        <v>231693534.023588</v>
+        <v>579233835.05897</v>
       </c>
       <c r="S26" s="54" t="n">
         <f aca="false">S23*$C$11</f>
-        <v>241267324.992527</v>
+        <v>603168312.481316</v>
       </c>
       <c r="T26" s="54" t="n">
         <f aca="false">T23*$C$11</f>
-        <v>250410295.367863</v>
+        <v>626025738.419657</v>
       </c>
       <c r="U26" s="54" t="n">
         <f aca="false">U23*$C$11</f>
-        <v>259141832.076309</v>
+        <v>647854580.190773</v>
       </c>
       <c r="V26" s="54" t="n">
         <f aca="false">V23*$C$11</f>
-        <v>267480449.632875</v>
+        <v>668701124.082188</v>
       </c>
       <c r="W26" s="54" t="n">
         <f aca="false">W23*$C$11</f>
-        <v>275443829.399396</v>
+        <v>688609573.498489</v>
       </c>
       <c r="X26" s="54" t="n">
         <f aca="false">X23*$C$11</f>
-        <v>283048857.076423</v>
+        <v>707622142.691057</v>
       </c>
       <c r="Y26" s="54" t="n">
         <f aca="false">Y23*$C$11</f>
-        <v>290311658.507984</v>
+        <v>725779146.269959</v>
       </c>
       <c r="Z26" s="54" t="n">
         <f aca="false">Z23*$C$11</f>
-        <v>297247633.875125</v>
+        <v>743119084.687811</v>
       </c>
       <c r="AA26" s="55" t="n">
         <f aca="false">SUM(C26:Z26)</f>
-        <v>4358411325.53902</v>
+        <v>10896028313.8475</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="8" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="C27" s="59" t="n">
         <f aca="false">C25-C26</f>
-        <v>12000000</v>
+        <v>30000000</v>
       </c>
       <c r="D27" s="59" t="n">
         <f aca="false">D25-D26</f>
-        <v>23460000</v>
+        <v>58650000</v>
       </c>
       <c r="E27" s="59" t="n">
         <f aca="false">E25-E26</f>
-        <v>34404300</v>
+        <v>86010750</v>
       </c>
       <c r="F27" s="59" t="n">
         <f aca="false">F25-F26</f>
-        <v>44856106.5</v>
+        <v>112140266.25</v>
       </c>
       <c r="G27" s="59" t="n">
         <f aca="false">G25-G26</f>
-        <v>54837581.7075</v>
+        <v>137093954.26875</v>
       </c>
       <c r="H27" s="59" t="n">
         <f aca="false">H25-H26</f>
-        <v>64369890.5306625</v>
+        <v>160924726.326656</v>
       </c>
       <c r="I27" s="59" t="n">
         <f aca="false">I25-I26</f>
-        <v>73473245.4567827</v>
+        <v>183683113.641957</v>
       </c>
       <c r="J27" s="59" t="n">
         <f aca="false">J25-J26</f>
-        <v>82166949.4112274</v>
+        <v>205417373.528069</v>
       </c>
       <c r="K27" s="59" t="n">
         <f aca="false">K25-K26</f>
-        <v>90469436.6877222</v>
+        <v>226173591.719306</v>
       </c>
       <c r="L27" s="59" t="n">
         <f aca="false">L25-L26</f>
-        <v>98398312.0367747</v>
+        <v>245995780.091937</v>
       </c>
       <c r="M27" s="59" t="n">
         <f aca="false">M25-M26</f>
-        <v>105970387.99512</v>
+        <v>264925969.9878</v>
       </c>
       <c r="N27" s="59" t="n">
         <f aca="false">N25-N26</f>
-        <v>113201720.535339</v>
+        <v>283004301.338349</v>
       </c>
       <c r="O27" s="59" t="n">
         <f aca="false">O25-O26</f>
-        <v>120107643.111249</v>
+        <v>300269107.778123</v>
       </c>
       <c r="P27" s="59" t="n">
         <f aca="false">P25-P26</f>
-        <v>126702799.171243</v>
+        <v>316756997.928107</v>
       </c>
       <c r="Q27" s="59" t="n">
         <f aca="false">Q25-Q26</f>
-        <v>133001173.208537</v>
+        <v>332502933.021343</v>
       </c>
       <c r="R27" s="59" t="n">
         <f aca="false">R25-R26</f>
-        <v>139016120.414153</v>
+        <v>347540301.035382</v>
       </c>
       <c r="S27" s="59" t="n">
         <f aca="false">S25-S26</f>
-        <v>144760394.995516</v>
+        <v>361900987.48879</v>
       </c>
       <c r="T27" s="59" t="n">
         <f aca="false">T25-T26</f>
-        <v>150246177.220718</v>
+        <v>375615443.051794</v>
       </c>
       <c r="U27" s="59" t="n">
         <f aca="false">U25-U26</f>
-        <v>155485099.245785</v>
+        <v>388712748.114464</v>
       </c>
       <c r="V27" s="59" t="n">
         <f aca="false">V25-V26</f>
-        <v>160488269.779725</v>
+        <v>401220674.449313</v>
       </c>
       <c r="W27" s="59" t="n">
         <f aca="false">W25-W26</f>
-        <v>165266297.639637</v>
+        <v>413165744.099093</v>
       </c>
       <c r="X27" s="59" t="n">
         <f aca="false">X25-X26</f>
-        <v>169829314.245854</v>
+        <v>424573285.614634</v>
       </c>
       <c r="Y27" s="59" t="n">
         <f aca="false">Y25-Y26</f>
-        <v>174186995.10479</v>
+        <v>435467487.761976</v>
       </c>
       <c r="Z27" s="59" t="n">
         <f aca="false">Z25-Z26</f>
-        <v>178348580.325075</v>
+        <v>445871450.812687</v>
       </c>
       <c r="AA27" s="55" t="n">
         <f aca="false">SUM(C27:Z27)</f>
-        <v>2615046795.32341</v>
+        <v>6537616988.30853</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="9" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="C28" s="54" t="n">
         <f aca="false">C22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="D28" s="54" t="n">
         <f aca="false">D22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="E28" s="54" t="n">
         <f aca="false">E22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="F28" s="54" t="n">
         <f aca="false">F22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="G28" s="54" t="n">
         <f aca="false">G22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="H28" s="54" t="n">
         <f aca="false">H22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="I28" s="54" t="n">
         <f aca="false">I22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="J28" s="54" t="n">
         <f aca="false">J22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="K28" s="54" t="n">
         <f aca="false">K22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="L28" s="54" t="n">
         <f aca="false">L22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="M28" s="54" t="n">
         <f aca="false">M22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="N28" s="54" t="n">
         <f aca="false">N22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="O28" s="54" t="n">
         <f aca="false">O22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="P28" s="54" t="n">
         <f aca="false">P22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="Q28" s="54" t="n">
         <f aca="false">Q22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="R28" s="54" t="n">
         <f aca="false">R22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="S28" s="54" t="n">
         <f aca="false">S22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="T28" s="54" t="n">
         <f aca="false">T22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="U28" s="54" t="n">
         <f aca="false">U22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="V28" s="54" t="n">
         <f aca="false">V22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="W28" s="54" t="n">
         <f aca="false">W22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="X28" s="54" t="n">
         <f aca="false">X22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="Y28" s="54" t="n">
         <f aca="false">Y22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="Z28" s="54" t="n">
         <f aca="false">Z22*$C$13</f>
-        <v>270000000</v>
+        <v>675000000</v>
       </c>
       <c r="AA28" s="55" t="n">
         <f aca="false">SUM(C28:Z28)</f>
-        <v>6480000000</v>
+        <v>16200000000</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="9" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="C29" s="54" t="n">
         <f aca="false">$C$14</f>
@@ -3996,318 +4126,318 @@
     </row>
     <row r="30" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="18" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C30" s="60" t="n">
         <f aca="false">C27-C28-C29</f>
-        <v>-398000000</v>
+        <v>-785000000</v>
       </c>
       <c r="D30" s="60" t="n">
         <f aca="false">D27-D28-D29</f>
-        <v>-386540000</v>
+        <v>-756350000</v>
       </c>
       <c r="E30" s="60" t="n">
         <f aca="false">E27-E28-E29</f>
-        <v>-375595700</v>
+        <v>-728989250</v>
       </c>
       <c r="F30" s="60" t="n">
         <f aca="false">F27-F28-F29</f>
-        <v>-365143893.5</v>
+        <v>-702859733.75</v>
       </c>
       <c r="G30" s="60" t="n">
         <f aca="false">G27-G28-G29</f>
-        <v>-355162418.2925</v>
+        <v>-677906045.73125</v>
       </c>
       <c r="H30" s="60" t="n">
         <f aca="false">H27-H28-H29</f>
-        <v>-345630109.469338</v>
+        <v>-654075273.673344</v>
       </c>
       <c r="I30" s="60" t="n">
         <f aca="false">I27-I28-I29</f>
-        <v>-336526754.543217</v>
+        <v>-631316886.358043</v>
       </c>
       <c r="J30" s="60" t="n">
         <f aca="false">J27-J28-J29</f>
-        <v>-327833050.588773</v>
+        <v>-609582626.471932</v>
       </c>
       <c r="K30" s="60" t="n">
         <f aca="false">K27-K28-K29</f>
-        <v>-319530563.312278</v>
+        <v>-588826408.280695</v>
       </c>
       <c r="L30" s="60" t="n">
         <f aca="false">L27-L28-L29</f>
-        <v>-311601687.963225</v>
+        <v>-569004219.908063</v>
       </c>
       <c r="M30" s="60" t="n">
         <f aca="false">M27-M28-M29</f>
-        <v>-304029612.00488</v>
+        <v>-550074030.0122</v>
       </c>
       <c r="N30" s="60" t="n">
         <f aca="false">N27-N28-N29</f>
-        <v>-296798279.464661</v>
+        <v>-531995698.661651</v>
       </c>
       <c r="O30" s="60" t="n">
         <f aca="false">O27-O28-O29</f>
-        <v>-289892356.888751</v>
+        <v>-514730892.221877</v>
       </c>
       <c r="P30" s="60" t="n">
         <f aca="false">P27-P28-P29</f>
-        <v>-283297200.828757</v>
+        <v>-498243002.071893</v>
       </c>
       <c r="Q30" s="60" t="n">
         <f aca="false">Q27-Q28-Q29</f>
-        <v>-276998826.791463</v>
+        <v>-482497066.978658</v>
       </c>
       <c r="R30" s="60" t="n">
         <f aca="false">R27-R28-R29</f>
-        <v>-270983879.585847</v>
+        <v>-467459698.964618</v>
       </c>
       <c r="S30" s="60" t="n">
         <f aca="false">S27-S28-S29</f>
-        <v>-265239605.004484</v>
+        <v>-453099012.51121</v>
       </c>
       <c r="T30" s="60" t="n">
         <f aca="false">T27-T28-T29</f>
-        <v>-259753822.779282</v>
+        <v>-439384556.948206</v>
       </c>
       <c r="U30" s="60" t="n">
         <f aca="false">U27-U28-U29</f>
-        <v>-254514900.754215</v>
+        <v>-426287251.885536</v>
       </c>
       <c r="V30" s="60" t="n">
         <f aca="false">V27-V28-V29</f>
-        <v>-249511730.220275</v>
+        <v>-413779325.550687</v>
       </c>
       <c r="W30" s="60" t="n">
         <f aca="false">W27-W28-W29</f>
-        <v>-244733702.360363</v>
+        <v>-401834255.900907</v>
       </c>
       <c r="X30" s="60" t="n">
         <f aca="false">X27-X28-X29</f>
-        <v>-240170685.754146</v>
+        <v>-390426714.385366</v>
       </c>
       <c r="Y30" s="60" t="n">
         <f aca="false">Y27-Y28-Y29</f>
-        <v>-235813004.89521</v>
+        <v>-379532512.238024</v>
       </c>
       <c r="Z30" s="60" t="n">
         <f aca="false">Z27-Z28-Z29</f>
-        <v>-231651419.674925</v>
+        <v>-369128549.187313</v>
       </c>
       <c r="AA30" s="61" t="n">
         <f aca="false">SUM(C30:Z30)</f>
-        <v>-7224953204.67659</v>
+        <v>-13022383011.6915</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="9" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="C32" s="54" t="n">
         <f aca="false">C30-$C$15</f>
-        <v>-1198000000</v>
+        <v>-1585000000</v>
       </c>
       <c r="D32" s="54" t="n">
         <f aca="false">D30</f>
-        <v>-386540000</v>
+        <v>-756350000</v>
       </c>
       <c r="E32" s="54" t="n">
         <f aca="false">E30</f>
-        <v>-375595700</v>
+        <v>-728989250</v>
       </c>
       <c r="F32" s="54" t="n">
         <f aca="false">F30</f>
-        <v>-365143893.5</v>
+        <v>-702859733.75</v>
       </c>
       <c r="G32" s="54" t="n">
         <f aca="false">G30</f>
-        <v>-355162418.2925</v>
+        <v>-677906045.73125</v>
       </c>
       <c r="H32" s="54" t="n">
         <f aca="false">H30</f>
-        <v>-345630109.469338</v>
+        <v>-654075273.673344</v>
       </c>
       <c r="I32" s="54" t="n">
         <f aca="false">I30</f>
-        <v>-336526754.543217</v>
+        <v>-631316886.358043</v>
       </c>
       <c r="J32" s="54" t="n">
         <f aca="false">J30</f>
-        <v>-327833050.588773</v>
+        <v>-609582626.471932</v>
       </c>
       <c r="K32" s="54" t="n">
         <f aca="false">K30</f>
-        <v>-319530563.312278</v>
+        <v>-588826408.280695</v>
       </c>
       <c r="L32" s="54" t="n">
         <f aca="false">L30</f>
-        <v>-311601687.963225</v>
+        <v>-569004219.908063</v>
       </c>
       <c r="M32" s="54" t="n">
         <f aca="false">M30</f>
-        <v>-304029612.00488</v>
+        <v>-550074030.0122</v>
       </c>
       <c r="N32" s="54" t="n">
         <f aca="false">N30</f>
-        <v>-296798279.464661</v>
+        <v>-531995698.661651</v>
       </c>
       <c r="O32" s="54" t="n">
         <f aca="false">O30</f>
-        <v>-289892356.888751</v>
+        <v>-514730892.221877</v>
       </c>
       <c r="P32" s="54" t="n">
         <f aca="false">P30</f>
-        <v>-283297200.828757</v>
+        <v>-498243002.071893</v>
       </c>
       <c r="Q32" s="54" t="n">
         <f aca="false">Q30</f>
-        <v>-276998826.791463</v>
+        <v>-482497066.978658</v>
       </c>
       <c r="R32" s="54" t="n">
         <f aca="false">R30</f>
-        <v>-270983879.585847</v>
+        <v>-467459698.964618</v>
       </c>
       <c r="S32" s="54" t="n">
         <f aca="false">S30</f>
-        <v>-265239605.004484</v>
+        <v>-453099012.51121</v>
       </c>
       <c r="T32" s="54" t="n">
         <f aca="false">T30</f>
-        <v>-259753822.779282</v>
+        <v>-439384556.948206</v>
       </c>
       <c r="U32" s="54" t="n">
         <f aca="false">U30</f>
-        <v>-254514900.754215</v>
+        <v>-426287251.885536</v>
       </c>
       <c r="V32" s="54" t="n">
         <f aca="false">V30</f>
-        <v>-249511730.220275</v>
+        <v>-413779325.550687</v>
       </c>
       <c r="W32" s="54" t="n">
         <f aca="false">W30</f>
-        <v>-244733702.360363</v>
+        <v>-401834255.900907</v>
       </c>
       <c r="X32" s="54" t="n">
         <f aca="false">X30</f>
-        <v>-240170685.754146</v>
+        <v>-390426714.385366</v>
       </c>
       <c r="Y32" s="54" t="n">
         <f aca="false">Y30</f>
-        <v>-235813004.89521</v>
+        <v>-379532512.238024</v>
       </c>
       <c r="Z32" s="54" t="n">
         <f aca="false">Z30</f>
-        <v>-231651419.674925</v>
+        <v>-369128549.187313</v>
       </c>
       <c r="AA32" s="55" t="n">
         <f aca="false">SUM(C32:Z32)</f>
-        <v>-8024953204.67659</v>
+        <v>-13822383011.6915</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="62" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="C33" s="63" t="n">
         <f aca="false">$C$16+C32</f>
-        <v>3802000000</v>
+        <v>8415000000</v>
       </c>
       <c r="D33" s="63" t="n">
         <f aca="false">C33+D32</f>
-        <v>3415460000</v>
+        <v>7658650000</v>
       </c>
       <c r="E33" s="63" t="n">
         <f aca="false">D33+E32</f>
-        <v>3039864300</v>
+        <v>6929660750</v>
       </c>
       <c r="F33" s="63" t="n">
         <f aca="false">E33+F32</f>
-        <v>2674720406.5</v>
+        <v>6226801016.25</v>
       </c>
       <c r="G33" s="63" t="n">
         <f aca="false">F33+G32</f>
-        <v>2319557988.2075</v>
+        <v>5548894970.51875</v>
       </c>
       <c r="H33" s="63" t="n">
         <f aca="false">G33+H32</f>
-        <v>1973927878.73816</v>
+        <v>4894819696.84541</v>
       </c>
       <c r="I33" s="63" t="n">
         <f aca="false">H33+I32</f>
-        <v>1637401124.19495</v>
+        <v>4263502810.48736</v>
       </c>
       <c r="J33" s="63" t="n">
         <f aca="false">I33+J32</f>
-        <v>1309568073.60617</v>
+        <v>3653920184.01543</v>
       </c>
       <c r="K33" s="63" t="n">
         <f aca="false">J33+K32</f>
-        <v>990037510.293895</v>
+        <v>3065093775.73474</v>
       </c>
       <c r="L33" s="63" t="n">
         <f aca="false">K33+L32</f>
-        <v>678435822.33067</v>
+        <v>2496089555.82667</v>
       </c>
       <c r="M33" s="63" t="n">
         <f aca="false">L33+M32</f>
-        <v>374406210.325789</v>
+        <v>1946015525.81447</v>
       </c>
       <c r="N33" s="63" t="n">
         <f aca="false">M33+N32</f>
-        <v>77607930.8611288</v>
+        <v>1414019827.15282</v>
       </c>
       <c r="O33" s="63" t="n">
         <f aca="false">N33+O32</f>
-        <v>-212284426.027622</v>
+        <v>899288934.930946</v>
       </c>
       <c r="P33" s="63" t="n">
         <f aca="false">O33+P32</f>
-        <v>-495581626.856379</v>
+        <v>401045932.859053</v>
       </c>
       <c r="Q33" s="63" t="n">
         <f aca="false">P33+Q32</f>
-        <v>-772580453.647842</v>
+        <v>-81451134.1196045</v>
       </c>
       <c r="R33" s="63" t="n">
         <f aca="false">Q33+R32</f>
-        <v>-1043564333.23369</v>
+        <v>-548910833.084222</v>
       </c>
       <c r="S33" s="63" t="n">
         <f aca="false">R33+S32</f>
-        <v>-1308803938.23817</v>
+        <v>-1002009845.59543</v>
       </c>
       <c r="T33" s="63" t="n">
         <f aca="false">S33+T32</f>
-        <v>-1568557761.01746</v>
+        <v>-1441394402.54364</v>
       </c>
       <c r="U33" s="63" t="n">
         <f aca="false">T33+U32</f>
-        <v>-1823072661.77167</v>
+        <v>-1867681654.42917</v>
       </c>
       <c r="V33" s="63" t="n">
         <f aca="false">U33+V32</f>
-        <v>-2072584391.99195</v>
+        <v>-2281460979.97986</v>
       </c>
       <c r="W33" s="63" t="n">
         <f aca="false">V33+W32</f>
-        <v>-2317318094.35231</v>
+        <v>-2683295235.88077</v>
       </c>
       <c r="X33" s="63" t="n">
         <f aca="false">W33+X32</f>
-        <v>-2557488780.10645</v>
+        <v>-3073721950.26613</v>
       </c>
       <c r="Y33" s="63" t="n">
         <f aca="false">X33+Y32</f>
-        <v>-2793301785.00166</v>
+        <v>-3453254462.50416</v>
       </c>
       <c r="Z33" s="63" t="n">
         <f aca="false">Y33+Z32</f>
-        <v>-3024953204.67659</v>
+        <v>-3822383011.69147</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="3" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
@@ -4320,11 +4450,11 @@
     </row>
     <row r="37" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="8" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="C37" s="64" t="n">
         <f aca="false">(NPV($C$17,D32:Z32)+C32)/1000000</f>
-        <v>-6806.91845762453</v>
+        <v>-11713.8346635723</v>
       </c>
       <c r="D37" s="46" t="str">
         <f aca="false">"(target: &gt; 0)"</f>
@@ -4333,7 +4463,7 @@
     </row>
     <row r="38" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="8" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="C38" s="65" t="n">
         <f aca="false">IFERROR((1+IRR(C32:Z32))^12-1,0)</f>
@@ -4346,7 +4476,7 @@
     </row>
     <row r="39" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="8" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C39" s="66" t="str">
         <f aca="false">IFERROR(MATCH(TRUE(),INDEX(C41:Z41&gt;=0,0),0),"&gt; 24")</f>
@@ -4359,11 +4489,11 @@
     </row>
     <row r="40" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="8" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="C40" s="66" t="n">
         <f aca="false">IFERROR(MATCH(TRUE(),INDEX(C33:Z33&lt;0,0),0)-1,"&gt;= 24")</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D40" s="46" t="str">
         <f aca="false">"(target: &gt;= 12)"</f>
@@ -4372,108 +4502,108 @@
     </row>
     <row r="41" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="67" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C41" s="68" t="n">
         <f aca="false">C32</f>
-        <v>-1198000000</v>
+        <v>-1585000000</v>
       </c>
       <c r="D41" s="68" t="n">
         <f aca="false">C41+D32</f>
-        <v>-1584540000</v>
+        <v>-2341350000</v>
       </c>
       <c r="E41" s="68" t="n">
         <f aca="false">D41+E32</f>
-        <v>-1960135700</v>
+        <v>-3070339250</v>
       </c>
       <c r="F41" s="68" t="n">
         <f aca="false">E41+F32</f>
-        <v>-2325279593.5</v>
+        <v>-3773198983.75</v>
       </c>
       <c r="G41" s="68" t="n">
         <f aca="false">F41+G32</f>
-        <v>-2680442011.7925</v>
+        <v>-4451105029.48125</v>
       </c>
       <c r="H41" s="68" t="n">
         <f aca="false">G41+H32</f>
-        <v>-3026072121.26184</v>
+        <v>-5105180303.15459</v>
       </c>
       <c r="I41" s="68" t="n">
         <f aca="false">H41+I32</f>
-        <v>-3362598875.80505</v>
+        <v>-5736497189.51264</v>
       </c>
       <c r="J41" s="68" t="n">
         <f aca="false">I41+J32</f>
-        <v>-3690431926.39383</v>
+        <v>-6346079815.98457</v>
       </c>
       <c r="K41" s="68" t="n">
         <f aca="false">J41+K32</f>
-        <v>-4009962489.70611</v>
+        <v>-6934906224.26526</v>
       </c>
       <c r="L41" s="68" t="n">
         <f aca="false">K41+L32</f>
-        <v>-4321564177.66933</v>
+        <v>-7503910444.17333</v>
       </c>
       <c r="M41" s="68" t="n">
         <f aca="false">L41+M32</f>
-        <v>-4625593789.67421</v>
+        <v>-8053984474.18553</v>
       </c>
       <c r="N41" s="68" t="n">
         <f aca="false">M41+N32</f>
-        <v>-4922392069.13887</v>
+        <v>-8585980172.84718</v>
       </c>
       <c r="O41" s="68" t="n">
         <f aca="false">N41+O32</f>
-        <v>-5212284426.02762</v>
+        <v>-9100711065.06905</v>
       </c>
       <c r="P41" s="68" t="n">
         <f aca="false">O41+P32</f>
-        <v>-5495581626.85638</v>
+        <v>-9598954067.14095</v>
       </c>
       <c r="Q41" s="68" t="n">
         <f aca="false">P41+Q32</f>
-        <v>-5772580453.64784</v>
+        <v>-10081451134.1196</v>
       </c>
       <c r="R41" s="68" t="n">
         <f aca="false">Q41+R32</f>
-        <v>-6043564333.23369</v>
+        <v>-10548910833.0842</v>
       </c>
       <c r="S41" s="68" t="n">
         <f aca="false">R41+S32</f>
-        <v>-6308803938.23817</v>
+        <v>-11002009845.5954</v>
       </c>
       <c r="T41" s="68" t="n">
         <f aca="false">S41+T32</f>
-        <v>-6568557761.01746</v>
+        <v>-11441394402.5436</v>
       </c>
       <c r="U41" s="68" t="n">
         <f aca="false">T41+U32</f>
-        <v>-6823072661.77167</v>
+        <v>-11867681654.4292</v>
       </c>
       <c r="V41" s="68" t="n">
         <f aca="false">U41+V32</f>
-        <v>-7072584391.99195</v>
+        <v>-12281460979.9799</v>
       </c>
       <c r="W41" s="68" t="n">
         <f aca="false">V41+W32</f>
-        <v>-7317318094.35231</v>
+        <v>-12683295235.8808</v>
       </c>
       <c r="X41" s="68" t="n">
         <f aca="false">W41+X32</f>
-        <v>-7557488780.10646</v>
+        <v>-13073721950.2661</v>
       </c>
       <c r="Y41" s="68" t="n">
         <f aca="false">X41+Y32</f>
-        <v>-7793301785.00166</v>
+        <v>-13453254462.5042</v>
       </c>
       <c r="Z41" s="68" t="n">
         <f aca="false">Y41+Z32</f>
-        <v>-8024953204.67659</v>
+        <v>-13822383011.6915</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="3" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
@@ -4486,7 +4616,7 @@
     </row>
     <row r="44" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="8" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="C44" s="69" t="str">
         <f aca="false">IF(AND(C37&gt;0,C38&gt;CHOOSE($C$6,'1. Assumptions'!C35,'1. Assumptions'!D35,'1. Assumptions'!E35)),"✓ GO — NPV+ và IRR &gt; WACC",IF(C37&lt;0,"✗ NO-GO — NPV âm: dự án không tạo giá trị","⚠ HOLD — IRR thấp hơn kỳ vọng, cần điều chỉnh"))</f>
@@ -4652,8 +4782,8 @@
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="2" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>

<commit_message>
docs: strengthen Decision Note with benchmarks and hidden costs
</commit_message>
<xml_diff>
--- a/2A202601912_HuynhThiHaiChau_Day24.xlsx
+++ b/2A202601912_HuynhThiHaiChau_Day24.xlsx
@@ -33,6 +33,39 @@
     <author>Huỳnh Thị Hải Châu</author>
   </authors>
   <commentList>
+    <comment ref="B39" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Pricing benchmark: Intercom lists $29 per seat/month plus $0.99 per Fin AI outcome. https://www.intercom.com/ai-chatbot | Unit economics benchmark: Bessemer recommends CLTV/CAC 3x+ and SMB CAC payback under 12 months. https://www.bvp.com/assets/uploads/2021/09/scaling-to-100-million-by-mary-d-onofrio.pdf</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>57</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>-197</xdr:colOff>
+                <xdr:row>1</xdr:row>
+                <xdr:rowOff>19</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
     <comment ref="D7" authorId="0">
       <text>
         <r>
@@ -496,7 +529,9 @@
     <t xml:space="preserve">8. Decision Note  /  Ghi chú quyết định</t>
   </si>
   <si>
-    <t xml:space="preserve">ViVi dùng hybrid pricing B2B: phí nền tảng 9 triệu VND/showroom/tháng cộng usage bình quân 1,5 triệu, nên ARPU Base là 10,5 triệu. TAM dùng cho bài là 10.000 điểm bán ô tô tại Đông Nam Á; mạng lưới VinFast là nhóm khách hàng đầu tiên. Adoption 0,3%/tháng ở Base tương đương 30 điểm bán mới. Với gross margin 61,9%, LTV/CAC đạt 4,81x và payback 6,9 tháng. Pessimistic hạ adoption còn 0,1%, tăng churn và CAC lên 1,5x Base; 10 tỷ VND tiền mặt giữ runway 14 tháng để nhóm có thời gian cắt scope.</t>
+    <t xml:space="preserve">ViVi dùng hybrid B2B: 9 triệu đồng phí nền tảng/showroom/tháng cộng 1,5 triệu đồng usage, nên ARPU Base là 10,5 triệu đồng. Cách thu này bám logic Intercom: gói nền tảng từ 29 USD/seat/tháng và Fin AI Agent thêm 0,99 USD cho mỗi outcome. Với ViVi, phí nền tảng chi trả cho tích hợp dữ liệu xe, lịch lái thử và dashboard; phần usage hấp thụ biến động hội thoại. CAC Base 45 triệu đồng được ước tính bottom-up từ demo, tích hợp, onboarding và hỗ trợ bán hàng B2B. Kết quả payback 6,9 tháng, thấp hơn mốc 12 tháng dành cho SMB theo Bessemer.
+Ngoài API 1,5 triệu và hạ tầng 1,2 triệu đồng/showroom/tháng, tôi dành 1,3 triệu đồng cho AI hidden costs, bằng 86,7% API cost. Mỗi tuần nhóm lấy mẫu lỗi và gắn nhãn lại intent; mỗi tháng cập nhật knowledge base; mỗi quý chạy regression test rồi chỉnh prompt hoặc retrain. PM giữ rubric, kỹ sư vận hành pipeline, còn sales ops kiểm tra thủ công các ca có giá, khuyến mại hoặc booking bất thường. Khoản này gắn với công việc cụ thể, không phải buffer chung.
+Ở Base, gross margin là 61,9%, LTV/CAC đạt 4,81x, CAC payback là 6,9 tháng, NPV dương và dự án hoàn vốn ở tháng 18. Pessimistic hạ ARPU còn 8 triệu đồng, adoption còn 0,1%, churn lên 4,5% và CAC lên 67,5 triệu đồng; NPV khi đó âm. Với 10 tỷ đồng tiền mặt, runway vẫn đạt 14 tháng. Nếu kết quả thực tế bám kịch bản này ba tháng liên tiếp, nhóm sẽ dừng rollout mới, đặt trần usage, dùng model rẻ hơn cho tác vụ ít rủi ro, giữ human QA cho ca quan trọng và chốt vốn trước khi runway xuống dưới 12 tháng.</t>
   </si>
   <si>
     <t xml:space="preserve">Tab 2 — UNIT ECONOMICS  /  Kinh tế đơn vị</t>
@@ -941,8 +976,8 @@
     </font>
     <font>
       <i val="true"/>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -2287,7 +2322,7 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="24" t="s">
         <v>53</v>
       </c>
@@ -2296,14 +2331,14 @@
       <c r="E39" s="24"/>
       <c r="F39" s="24"/>
     </row>
-    <row r="40" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="24"/>
       <c r="C40" s="24"/>
       <c r="D40" s="24"/>
       <c r="E40" s="24"/>
       <c r="F40" s="24"/>
     </row>
-    <row r="41" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="24"/>
       <c r="C41" s="24"/>
       <c r="D41" s="24"/>

</xml_diff>